<commit_message>
dados do 2Q2026 da AVGO
</commit_message>
<xml_diff>
--- a/analise_eua/semicondutores/broadcom/avgo_indicators.xlsx
+++ b/analise_eua/semicondutores/broadcom/avgo_indicators.xlsx
@@ -21,13 +21,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -46,13 +49,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,166 +436,166 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>P/L Damodaran</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>P/L</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>L/P</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Margem Líquida</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>P/VPA</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valor de Mercado</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Dívida Bruta</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Caixa e Equivalentes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/EBITDA</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/PL</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ROE</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ROIC</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>FCO</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>FCI</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>FCF</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Free Cash Flow</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Capex</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Net Capex</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>R&amp;D</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Adj Net Capex</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Working Capital</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Reinvestment Rate</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>FCFE</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>DPA</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Payout</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Buyback</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>2025</v>
       </c>
       <c r="B2" t="n">
-        <v>81.95</v>
+        <v>81.78</v>
       </c>
       <c r="C2" t="n">
-        <v>81.91</v>
+        <v>81.73999999999999</v>
       </c>
       <c r="D2" t="n">
         <v>1.22</v>
@@ -593,10 +607,10 @@
         <v>36.2</v>
       </c>
       <c r="G2" t="n">
-        <v>23.32</v>
+        <v>23.27</v>
       </c>
       <c r="H2" t="n">
-        <v>1895119280</v>
+        <v>1891161200</v>
       </c>
       <c r="I2" t="n">
         <v>65136</v>
@@ -614,7 +628,7 @@
         <v>0.6</v>
       </c>
       <c r="N2" t="n">
-        <v>74.61</v>
+        <v>74.45</v>
       </c>
       <c r="O2" t="n">
         <v>28.45</v>
@@ -669,14 +683,14 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>2024</v>
       </c>
       <c r="B3" t="n">
-        <v>125.66</v>
+        <v>125.39</v>
       </c>
       <c r="C3" t="n">
-        <v>126.14</v>
+        <v>125.87</v>
       </c>
       <c r="D3" t="n">
         <v>0.79</v>
@@ -688,10 +702,10 @@
         <v>11.43</v>
       </c>
       <c r="G3" t="n">
-        <v>10.94</v>
+        <v>10.92</v>
       </c>
       <c r="H3" t="n">
-        <v>740764799.9999999</v>
+        <v>739192640</v>
       </c>
       <c r="I3" t="n">
         <v>67566</v>
@@ -709,7 +723,7 @@
         <v>0.86</v>
       </c>
       <c r="N3" t="n">
-        <v>56.84</v>
+        <v>56.73</v>
       </c>
       <c r="O3" t="n">
         <v>8.710000000000001</v>
@@ -764,14 +778,14 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>2023</v>
       </c>
       <c r="B4" t="n">
-        <v>26.56</v>
+        <v>26.5</v>
       </c>
       <c r="C4" t="n">
-        <v>26.56</v>
+        <v>26.5</v>
       </c>
       <c r="D4" t="n">
         <v>3.77</v>
@@ -783,10 +797,10 @@
         <v>39.31</v>
       </c>
       <c r="G4" t="n">
-        <v>15.59</v>
+        <v>15.56</v>
       </c>
       <c r="H4" t="n">
-        <v>373956500</v>
+        <v>373168000</v>
       </c>
       <c r="I4" t="n">
         <v>39229</v>
@@ -804,7 +818,7 @@
         <v>1.04</v>
       </c>
       <c r="N4" t="n">
-        <v>23.88</v>
+        <v>23.83</v>
       </c>
       <c r="O4" t="n">
         <v>58.7</v>
@@ -859,17 +873,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="1" t="n">
         <v>2022</v>
       </c>
       <c r="B5" t="n">
-        <v>19.04</v>
+        <v>19</v>
       </c>
       <c r="C5" t="n">
-        <v>19.04</v>
+        <v>19</v>
       </c>
       <c r="D5" t="n">
-        <v>5.25</v>
+        <v>5.26</v>
       </c>
       <c r="E5" t="n">
         <v>14754</v>
@@ -878,10 +892,10 @@
         <v>33.8</v>
       </c>
       <c r="G5" t="n">
-        <v>9.41</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>213702500</v>
+        <v>213252600</v>
       </c>
       <c r="I5" t="n">
         <v>39515</v>
@@ -899,7 +913,7 @@
         <v>1.19</v>
       </c>
       <c r="N5" t="n">
-        <v>16.32</v>
+        <v>16.29</v>
       </c>
       <c r="O5" t="n">
         <v>49.42</v>
@@ -954,17 +968,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="1" t="n">
         <v>2021</v>
       </c>
       <c r="B6" t="n">
-        <v>32.46</v>
+        <v>32.39</v>
       </c>
       <c r="C6" t="n">
-        <v>32.46</v>
+        <v>32.39</v>
       </c>
       <c r="D6" t="n">
-        <v>3.08</v>
+        <v>3.09</v>
       </c>
       <c r="E6" t="n">
         <v>9058</v>
@@ -973,10 +987,10 @@
         <v>23.45</v>
       </c>
       <c r="G6" t="n">
-        <v>8.369999999999999</v>
+        <v>8.35</v>
       </c>
       <c r="H6" t="n">
-        <v>208936000</v>
+        <v>208526000</v>
       </c>
       <c r="I6" t="n">
         <v>39730</v>
@@ -994,7 +1008,7 @@
         <v>1.1</v>
       </c>
       <c r="N6" t="n">
-        <v>26.11</v>
+        <v>26.06</v>
       </c>
       <c r="O6" t="n">
         <v>25.79</v>
@@ -1049,14 +1063,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="1" t="n">
         <v>2020</v>
       </c>
       <c r="B7" t="n">
-        <v>54.07</v>
+        <v>53.97</v>
       </c>
       <c r="C7" t="n">
-        <v>54.11</v>
+        <v>54</v>
       </c>
       <c r="D7" t="n">
         <v>1.85</v>
@@ -1068,10 +1082,10 @@
         <v>11.15</v>
       </c>
       <c r="G7" t="n">
-        <v>6.03</v>
+        <v>6.02</v>
       </c>
       <c r="H7" t="n">
-        <v>143996400</v>
+        <v>143715000</v>
       </c>
       <c r="I7" t="n">
         <v>41062</v>
@@ -1089,7 +1103,7 @@
         <v>1.4</v>
       </c>
       <c r="N7" t="n">
-        <v>38.71</v>
+        <v>38.65</v>
       </c>
       <c r="O7" t="n">
         <v>11.15</v>
@@ -1144,17 +1158,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="1" t="n">
         <v>2019</v>
       </c>
       <c r="B8" t="n">
-        <v>39.77</v>
+        <v>39.68</v>
       </c>
       <c r="C8" t="n">
-        <v>39.78</v>
+        <v>39.69</v>
       </c>
       <c r="D8" t="n">
-        <v>2.51</v>
+        <v>2.52</v>
       </c>
       <c r="E8" t="n">
         <v>4013</v>
@@ -1163,10 +1177,10 @@
         <v>11.93</v>
       </c>
       <c r="G8" t="n">
-        <v>4.3</v>
+        <v>4.29</v>
       </c>
       <c r="H8" t="n">
-        <v>107181400</v>
+        <v>106942600</v>
       </c>
       <c r="I8" t="n">
         <v>32798</v>
@@ -1184,7 +1198,7 @@
         <v>1.11</v>
       </c>
       <c r="N8" t="n">
-        <v>33.62</v>
+        <v>33.56</v>
       </c>
       <c r="O8" t="n">
         <v>10.81</v>
@@ -1239,17 +1253,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="1" t="n">
         <v>2018</v>
       </c>
       <c r="B9" t="n">
-        <v>6.64</v>
+        <v>6.62</v>
       </c>
       <c r="C9" t="n">
-        <v>6.63</v>
+        <v>6.62</v>
       </c>
       <c r="D9" t="n">
-        <v>15.07</v>
+        <v>15.1</v>
       </c>
       <c r="E9" t="n">
         <v>5650</v>
@@ -1261,7 +1275,7 @@
         <v>3.05</v>
       </c>
       <c r="H9" t="n">
-        <v>81342800</v>
+        <v>81175600</v>
       </c>
       <c r="I9" t="n">
         <v>17493</v>
@@ -1279,7 +1293,7 @@
         <v>0.5</v>
       </c>
       <c r="N9" t="n">
-        <v>16.73</v>
+        <v>16.7</v>
       </c>
       <c r="O9" t="n">
         <v>45.99</v>
@@ -1334,17 +1348,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="1" t="n">
         <v>2017</v>
       </c>
       <c r="B10" t="n">
-        <v>52.3</v>
+        <v>52.2</v>
       </c>
       <c r="C10" t="n">
-        <v>52.27</v>
+        <v>52.18</v>
       </c>
       <c r="D10" t="n">
-        <v>1.91</v>
+        <v>1.92</v>
       </c>
       <c r="E10" t="n">
         <v>2834</v>
@@ -1353,10 +1367,10 @@
         <v>9.59</v>
       </c>
       <c r="G10" t="n">
-        <v>3.82</v>
+        <v>3.81</v>
       </c>
       <c r="H10" t="n">
-        <v>88492500</v>
+        <v>88330500</v>
       </c>
       <c r="I10" t="n">
         <v>17548</v>
@@ -1374,7 +1388,7 @@
         <v>0.27</v>
       </c>
       <c r="N10" t="n">
-        <v>33.46</v>
+        <v>33.41</v>
       </c>
       <c r="O10" t="n">
         <v>7.3</v>
@@ -1439,1678 +1453,1773 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE17"/>
+  <dimension ref="A1:AE18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>P/L Damodaran</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>P/L</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>L/P</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Margem Líquida</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>P/VPA</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valor de Mercado</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Dívida Bruta</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Caixa e Equivalentes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/EBITDA</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/PL</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ROE</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ROIC</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>FCO</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>FCI</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>FCF</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Free Cash Flow</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Capex</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Net Capex</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>R&amp;D</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Adj Net Capex</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Working Capital</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Reinvestment Rate</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>FCFE</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>DPA</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Payout</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Buyback</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46054</v>
+      <c r="A2" s="2" t="n">
+        <v>46143</v>
       </c>
       <c r="B2" t="n">
-        <v>206.15</v>
+        <v>227.8</v>
       </c>
       <c r="C2" t="n">
-        <v>68.72</v>
+        <v>82.13</v>
       </c>
       <c r="D2" t="n">
-        <v>1.46</v>
+        <v>1.22</v>
       </c>
       <c r="E2" t="n">
-        <v>8713</v>
+        <v>10951</v>
       </c>
       <c r="F2" t="n">
-        <v>38.06</v>
+        <v>41.96</v>
       </c>
       <c r="G2" t="n">
-        <v>18.96</v>
+        <v>24.19</v>
       </c>
       <c r="H2" t="n">
-        <v>1514986550</v>
+        <v>2120817190</v>
       </c>
       <c r="I2" t="n">
-        <v>66057</v>
+        <v>64907</v>
       </c>
       <c r="J2" t="n">
-        <v>14174</v>
+        <v>19628</v>
       </c>
       <c r="K2" t="n">
-        <v>51883</v>
+        <v>45279</v>
       </c>
       <c r="L2" t="n">
-        <v>1.91</v>
+        <v>1.43</v>
       </c>
       <c r="M2" t="n">
-        <v>0.65</v>
+        <v>0.52</v>
       </c>
       <c r="N2" t="n">
-        <v>57.79</v>
+        <v>68.41</v>
       </c>
       <c r="O2" t="n">
-        <v>27.49</v>
+        <v>29.38</v>
       </c>
       <c r="P2" t="n">
-        <v>16.75</v>
+        <v>18.44</v>
       </c>
       <c r="Q2" t="n">
-        <v>8260</v>
+        <v>10493</v>
       </c>
       <c r="R2" t="n">
-        <v>-115</v>
+        <v>-208</v>
       </c>
       <c r="S2" t="n">
-        <v>-10149</v>
+        <v>-4831</v>
       </c>
       <c r="T2" t="n">
-        <v>8010</v>
+        <v>10262</v>
       </c>
       <c r="U2" t="n">
-        <v>250</v>
+        <v>231</v>
       </c>
       <c r="V2" t="n">
-        <v>60</v>
+        <v>170</v>
       </c>
       <c r="W2" t="n">
-        <v>2965</v>
+        <v>2995</v>
       </c>
       <c r="X2" t="n">
-        <v>11021</v>
+        <v>11873</v>
       </c>
       <c r="Y2" t="n">
-        <v>15203</v>
+        <v>23351</v>
       </c>
       <c r="Z2" t="n">
-        <v>59.66</v>
+        <v>53.48</v>
       </c>
       <c r="AA2" t="n">
-        <v>15016</v>
+        <v>22952</v>
       </c>
       <c r="AB2" t="n">
-        <v>20179</v>
+        <v>25207</v>
       </c>
       <c r="AC2" t="n">
         <v>0.65</v>
       </c>
       <c r="AD2" t="n">
-        <v>41.99</v>
+        <v>33.21</v>
       </c>
       <c r="AE2" t="n">
-        <v>7850</v>
+        <v>600</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>45870</v>
+      <c r="A3" s="2" t="n">
+        <v>46054</v>
       </c>
       <c r="B3" t="n">
-        <v>337.39</v>
+        <v>205.72</v>
       </c>
       <c r="C3" t="n">
-        <v>109.74</v>
+        <v>68.58</v>
       </c>
       <c r="D3" t="n">
-        <v>0.91</v>
+        <v>1.46</v>
       </c>
       <c r="E3" t="n">
-        <v>6029</v>
+        <v>8713</v>
       </c>
       <c r="F3" t="n">
-        <v>25.95</v>
+        <v>38.06</v>
       </c>
       <c r="G3" t="n">
-        <v>19.07</v>
+        <v>18.92</v>
       </c>
       <c r="H3" t="n">
-        <v>1396805340</v>
+        <v>1511810080</v>
       </c>
       <c r="I3" t="n">
-        <v>64229</v>
+        <v>66057</v>
       </c>
       <c r="J3" t="n">
-        <v>10718</v>
+        <v>14174</v>
       </c>
       <c r="K3" t="n">
-        <v>53511</v>
+        <v>51883</v>
       </c>
       <c r="L3" t="n">
-        <v>2.4</v>
+        <v>1.91</v>
       </c>
       <c r="M3" t="n">
-        <v>0.73</v>
+        <v>0.65</v>
       </c>
       <c r="N3" t="n">
-        <v>64.92</v>
+        <v>57.67</v>
       </c>
       <c r="O3" t="n">
-        <v>17.38</v>
+        <v>27.49</v>
       </c>
       <c r="P3" t="n">
-        <v>11.84</v>
+        <v>16.75</v>
       </c>
       <c r="Q3" t="n">
-        <v>7166</v>
+        <v>8260</v>
       </c>
       <c r="R3" t="n">
-        <v>94</v>
+        <v>-115</v>
       </c>
       <c r="S3" t="n">
-        <v>-6014</v>
+        <v>-10149</v>
       </c>
       <c r="T3" t="n">
-        <v>7024</v>
+        <v>8010</v>
       </c>
       <c r="U3" t="n">
-        <v>142</v>
+        <v>250</v>
       </c>
       <c r="V3" t="n">
-        <v>-17</v>
+        <v>60</v>
       </c>
       <c r="W3" t="n">
-        <v>3050</v>
+        <v>2965</v>
       </c>
       <c r="X3" t="n">
-        <v>10332</v>
+        <v>11021</v>
       </c>
       <c r="Y3" t="n">
-        <v>8294</v>
+        <v>15203</v>
       </c>
       <c r="Z3" t="n">
-        <v>73.38</v>
+        <v>59.66</v>
       </c>
       <c r="AA3" t="n">
-        <v>2768</v>
+        <v>15016</v>
       </c>
       <c r="AB3" t="n">
-        <v>15456</v>
+        <v>20179</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.59</v>
+        <v>0.65</v>
       </c>
       <c r="AD3" t="n">
-        <v>67.29000000000001</v>
+        <v>41.99</v>
       </c>
       <c r="AE3" t="n">
-        <v>0</v>
+        <v>7850</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>45778</v>
+      <c r="A4" s="2" t="n">
+        <v>45870</v>
       </c>
       <c r="B4" t="n">
-        <v>228.13</v>
+        <v>336.69</v>
       </c>
       <c r="C4" t="n">
-        <v>37.72</v>
+        <v>109.51</v>
       </c>
       <c r="D4" t="n">
-        <v>2.65</v>
+        <v>0.91</v>
       </c>
       <c r="E4" t="n">
-        <v>5971</v>
+        <v>6029</v>
       </c>
       <c r="F4" t="n">
-        <v>33.09</v>
+        <v>25.95</v>
       </c>
       <c r="G4" t="n">
-        <v>16.28</v>
+        <v>19.03</v>
       </c>
       <c r="H4" t="n">
-        <v>1132645410</v>
+        <v>1393882660</v>
       </c>
       <c r="I4" t="n">
-        <v>67282</v>
+        <v>64229</v>
       </c>
       <c r="J4" t="n">
-        <v>9472</v>
+        <v>10718</v>
       </c>
       <c r="K4" t="n">
-        <v>57810</v>
+        <v>53511</v>
       </c>
       <c r="L4" t="n">
-        <v>2.98</v>
+        <v>2.4</v>
       </c>
       <c r="M4" t="n">
-        <v>0.83</v>
+        <v>0.73</v>
       </c>
       <c r="N4" t="n">
-        <v>61.29</v>
+        <v>64.79000000000001</v>
       </c>
       <c r="O4" t="n">
-        <v>15.4</v>
+        <v>17.38</v>
       </c>
       <c r="P4" t="n">
-        <v>10.68</v>
+        <v>11.84</v>
       </c>
       <c r="Q4" t="n">
-        <v>6555</v>
+        <v>7166</v>
       </c>
       <c r="R4" t="n">
-        <v>-133</v>
+        <v>94</v>
       </c>
       <c r="S4" t="n">
-        <v>-6257</v>
+        <v>-6014</v>
       </c>
       <c r="T4" t="n">
-        <v>6411</v>
+        <v>7024</v>
       </c>
       <c r="U4" t="n">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="V4" t="n">
-        <v>-34</v>
+        <v>-17</v>
       </c>
       <c r="W4" t="n">
-        <v>2693</v>
+        <v>3050</v>
       </c>
       <c r="X4" t="n">
-        <v>9680</v>
+        <v>10332</v>
       </c>
       <c r="Y4" t="n">
-        <v>1584</v>
+        <v>8294</v>
       </c>
       <c r="Z4" t="n">
-        <v>83.22</v>
+        <v>73.38</v>
       </c>
       <c r="AA4" t="n">
-        <v>-2315</v>
+        <v>2768</v>
       </c>
       <c r="AB4" t="n">
-        <v>15950</v>
+        <v>15456</v>
       </c>
       <c r="AC4" t="n">
         <v>0.59</v>
       </c>
       <c r="AD4" t="n">
-        <v>56.09</v>
+        <v>67.29000000000001</v>
       </c>
       <c r="AE4" t="n">
-        <v>2450</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>45689</v>
+      <c r="A5" s="2" t="n">
+        <v>45778</v>
       </c>
       <c r="B5" t="n">
-        <v>168.62</v>
+        <v>227.64</v>
       </c>
       <c r="C5" t="n">
-        <v>23.93</v>
+        <v>37.64</v>
       </c>
       <c r="D5" t="n">
-        <v>4.18</v>
+        <v>2.66</v>
       </c>
       <c r="E5" t="n">
-        <v>6402</v>
+        <v>5971</v>
       </c>
       <c r="F5" t="n">
-        <v>36.89</v>
+        <v>33.09</v>
       </c>
       <c r="G5" t="n">
-        <v>13.3</v>
+        <v>16.25</v>
       </c>
       <c r="H5" t="n">
-        <v>927919799.9999999</v>
+        <v>1130244840</v>
       </c>
       <c r="I5" t="n">
-        <v>66579</v>
+        <v>67282</v>
       </c>
       <c r="J5" t="n">
-        <v>9307</v>
+        <v>9472</v>
       </c>
       <c r="K5" t="n">
-        <v>57272</v>
+        <v>57810</v>
       </c>
       <c r="L5" t="n">
-        <v>3.65</v>
+        <v>2.98</v>
       </c>
       <c r="M5" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="N5" t="n">
-        <v>62.85</v>
+        <v>61.16</v>
       </c>
       <c r="O5" t="n">
-        <v>10.14</v>
+        <v>15.4</v>
       </c>
       <c r="P5" t="n">
-        <v>8.01</v>
+        <v>10.68</v>
       </c>
       <c r="Q5" t="n">
-        <v>6113</v>
+        <v>6555</v>
       </c>
       <c r="R5" t="n">
-        <v>-174</v>
+        <v>-133</v>
       </c>
       <c r="S5" t="n">
-        <v>-5980</v>
+        <v>-6257</v>
       </c>
       <c r="T5" t="n">
-        <v>6013</v>
+        <v>6411</v>
       </c>
       <c r="U5" t="n">
-        <v>100</v>
+        <v>144</v>
       </c>
       <c r="V5" t="n">
-        <v>-53</v>
+        <v>-34</v>
       </c>
       <c r="W5" t="n">
-        <v>2253</v>
+        <v>2693</v>
       </c>
       <c r="X5" t="n">
-        <v>9276</v>
+        <v>9680</v>
       </c>
       <c r="Y5" t="n">
-        <v>80</v>
+        <v>1584</v>
       </c>
       <c r="Z5" t="n">
-        <v>112.86</v>
+        <v>83.22</v>
       </c>
       <c r="AA5" t="n">
-        <v>21825</v>
+        <v>-2315</v>
       </c>
       <c r="AB5" t="n">
-        <v>12102</v>
+        <v>15950</v>
       </c>
       <c r="AC5" t="n">
         <v>0.59</v>
       </c>
       <c r="AD5" t="n">
-        <v>50.41</v>
+        <v>56.09</v>
       </c>
       <c r="AE5" t="n">
-        <v>0</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>45505</v>
+      <c r="A6" s="2" t="n">
+        <v>45689</v>
       </c>
       <c r="B6" t="n">
-        <v>-398.9</v>
+        <v>168.27</v>
       </c>
       <c r="C6" t="n">
-        <v>10.63</v>
+        <v>23.88</v>
       </c>
       <c r="D6" t="n">
-        <v>9.41</v>
+        <v>4.19</v>
       </c>
       <c r="E6" t="n">
-        <v>3937</v>
+        <v>6402</v>
       </c>
       <c r="F6" t="n">
-        <v>-14.34</v>
+        <v>36.89</v>
       </c>
       <c r="G6" t="n">
-        <v>11.39</v>
+        <v>13.27</v>
       </c>
       <c r="H6" t="n">
-        <v>747945200.0000001</v>
+        <v>925994850</v>
       </c>
       <c r="I6" t="n">
-        <v>66798</v>
+        <v>66579</v>
       </c>
       <c r="J6" t="n">
-        <v>9952</v>
+        <v>9307</v>
       </c>
       <c r="K6" t="n">
-        <v>56846</v>
+        <v>57272</v>
       </c>
       <c r="L6" t="n">
-        <v>4.29</v>
+        <v>3.65</v>
       </c>
       <c r="M6" t="n">
-        <v>0.87</v>
+        <v>0.82</v>
       </c>
       <c r="N6" t="n">
-        <v>60.73</v>
+        <v>62.73</v>
       </c>
       <c r="O6" t="n">
-        <v>7.42</v>
+        <v>10.14</v>
       </c>
       <c r="P6" t="n">
-        <v>6.21</v>
+        <v>8.01</v>
       </c>
       <c r="Q6" t="n">
-        <v>4963</v>
+        <v>6113</v>
       </c>
       <c r="R6" t="n">
-        <v>3245</v>
+        <v>-174</v>
       </c>
       <c r="S6" t="n">
-        <v>-8065</v>
+        <v>-5980</v>
       </c>
       <c r="T6" t="n">
-        <v>4791</v>
+        <v>6013</v>
       </c>
       <c r="U6" t="n">
-        <v>172</v>
+        <v>100</v>
       </c>
       <c r="V6" t="n">
-        <v>-11</v>
+        <v>-53</v>
       </c>
       <c r="W6" t="n">
-        <v>2353</v>
+        <v>2253</v>
       </c>
       <c r="X6" t="n">
-        <v>8423</v>
+        <v>9276</v>
       </c>
       <c r="Y6" t="n">
-        <v>726</v>
+        <v>80</v>
       </c>
       <c r="Z6" t="n">
-        <v>71.11</v>
+        <v>112.86</v>
       </c>
       <c r="AA6" t="n">
-        <v>30304</v>
+        <v>21825</v>
       </c>
       <c r="AB6" t="n">
-        <v>-3896</v>
+        <v>12102</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.53</v>
+        <v>0.59</v>
       </c>
       <c r="AD6" t="n">
-        <v>-130.77</v>
+        <v>50.41</v>
       </c>
       <c r="AE6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>45413</v>
+      <c r="A7" s="2" t="n">
+        <v>45505</v>
       </c>
       <c r="B7" t="n">
-        <v>286.04</v>
+        <v>-398.08</v>
       </c>
       <c r="C7" t="n">
-        <v>54.64</v>
+        <v>10.61</v>
       </c>
       <c r="D7" t="n">
-        <v>1.83</v>
+        <v>9.43</v>
       </c>
       <c r="E7" t="n">
-        <v>3114</v>
+        <v>3937</v>
       </c>
       <c r="F7" t="n">
-        <v>16.99</v>
+        <v>-14.34</v>
       </c>
       <c r="G7" t="n">
-        <v>8.67</v>
+        <v>11.37</v>
       </c>
       <c r="H7" t="n">
-        <v>606685500</v>
+        <v>746406409.9999999</v>
       </c>
       <c r="I7" t="n">
-        <v>71590</v>
+        <v>66798</v>
       </c>
       <c r="J7" t="n">
-        <v>9809</v>
+        <v>9952</v>
       </c>
       <c r="K7" t="n">
-        <v>61781</v>
+        <v>56846</v>
       </c>
       <c r="L7" t="n">
-        <v>4.59</v>
+        <v>4.29</v>
       </c>
       <c r="M7" t="n">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="N7" t="n">
-        <v>49.7</v>
+        <v>60.62</v>
       </c>
       <c r="O7" t="n">
-        <v>14.62</v>
+        <v>7.42</v>
       </c>
       <c r="P7" t="n">
-        <v>8.800000000000001</v>
+        <v>6.21</v>
       </c>
       <c r="Q7" t="n">
-        <v>4580</v>
+        <v>4963</v>
       </c>
       <c r="R7" t="n">
-        <v>-706</v>
+        <v>3245</v>
       </c>
       <c r="S7" t="n">
-        <v>-5929</v>
+        <v>-8065</v>
       </c>
       <c r="T7" t="n">
-        <v>4448</v>
+        <v>4791</v>
       </c>
       <c r="U7" t="n">
-        <v>132</v>
+        <v>172</v>
       </c>
       <c r="V7" t="n">
-        <v>-41</v>
+        <v>-11</v>
       </c>
       <c r="W7" t="n">
-        <v>2415</v>
+        <v>2353</v>
       </c>
       <c r="X7" t="n">
-        <v>7352</v>
+        <v>8423</v>
       </c>
       <c r="Y7" t="n">
-        <v>5131</v>
+        <v>726</v>
       </c>
       <c r="Z7" t="n">
-        <v>73</v>
+        <v>71.11</v>
       </c>
       <c r="AA7" t="n">
-        <v>35608</v>
+        <v>30304</v>
       </c>
       <c r="AB7" t="n">
-        <v>11214</v>
+        <v>-3896</v>
       </c>
       <c r="AC7" t="n">
-        <v>5.25</v>
+        <v>0.53</v>
       </c>
       <c r="AD7" t="n">
-        <v>115.18</v>
+        <v>-130.77</v>
       </c>
       <c r="AE7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>45323</v>
+      <c r="A8" s="2" t="n">
+        <v>45413</v>
       </c>
       <c r="B8" t="n">
-        <v>433.82</v>
+        <v>285.45</v>
       </c>
       <c r="C8" t="n">
-        <v>44.86</v>
+        <v>54.52</v>
       </c>
       <c r="D8" t="n">
-        <v>2.23</v>
+        <v>1.83</v>
       </c>
       <c r="E8" t="n">
-        <v>2222</v>
+        <v>3114</v>
       </c>
       <c r="F8" t="n">
-        <v>11.08</v>
+        <v>16.99</v>
       </c>
       <c r="G8" t="n">
-        <v>8.18</v>
+        <v>8.65</v>
       </c>
       <c r="H8" t="n">
-        <v>574808400</v>
+        <v>605430000</v>
       </c>
       <c r="I8" t="n">
-        <v>73468</v>
+        <v>71590</v>
       </c>
       <c r="J8" t="n">
-        <v>11864</v>
+        <v>9809</v>
       </c>
       <c r="K8" t="n">
-        <v>61604</v>
+        <v>61781</v>
       </c>
       <c r="L8" t="n">
-        <v>4.23</v>
+        <v>4.59</v>
       </c>
       <c r="M8" t="n">
         <v>0.88</v>
       </c>
       <c r="N8" t="n">
-        <v>43.69</v>
+        <v>49.6</v>
       </c>
       <c r="O8" t="n">
-        <v>16.91</v>
+        <v>14.62</v>
       </c>
       <c r="P8" t="n">
-        <v>9.33</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="Q8" t="n">
-        <v>4815</v>
+        <v>4580</v>
       </c>
       <c r="R8" t="n">
-        <v>-25477</v>
+        <v>-706</v>
       </c>
       <c r="S8" t="n">
-        <v>18337</v>
+        <v>-5929</v>
       </c>
       <c r="T8" t="n">
-        <v>4693</v>
+        <v>4448</v>
       </c>
       <c r="U8" t="n">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="V8" t="n">
-        <v>-48</v>
+        <v>-41</v>
       </c>
       <c r="W8" t="n">
-        <v>2308</v>
+        <v>2415</v>
       </c>
       <c r="X8" t="n">
-        <v>6125</v>
+        <v>7352</v>
       </c>
       <c r="Y8" t="n">
-        <v>6823</v>
+        <v>5131</v>
       </c>
       <c r="Z8" t="n">
-        <v>49.98</v>
+        <v>73</v>
       </c>
       <c r="AA8" t="n">
-        <v>40170</v>
+        <v>35608</v>
       </c>
       <c r="AB8" t="n">
-        <v>12809</v>
+        <v>11214</v>
       </c>
       <c r="AC8" t="n">
-        <v>5.39</v>
+        <v>5.25</v>
       </c>
       <c r="AD8" t="n">
-        <v>183.77</v>
+        <v>115.18</v>
       </c>
       <c r="AE8" t="n">
-        <v>7176</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>45139</v>
+      <c r="A9" s="2" t="n">
+        <v>45323</v>
       </c>
       <c r="B9" t="n">
-        <v>111.72</v>
+        <v>432.93</v>
       </c>
       <c r="C9" t="n">
-        <v>27.22</v>
+        <v>44.77</v>
       </c>
       <c r="D9" t="n">
-        <v>3.67</v>
+        <v>2.23</v>
       </c>
       <c r="E9" t="n">
-        <v>3978</v>
+        <v>2222</v>
       </c>
       <c r="F9" t="n">
-        <v>37.21</v>
+        <v>11.08</v>
       </c>
       <c r="G9" t="n">
-        <v>16.71</v>
+        <v>8.16</v>
       </c>
       <c r="H9" t="n">
-        <v>369015500</v>
+        <v>573633200</v>
       </c>
       <c r="I9" t="n">
-        <v>38222</v>
+        <v>73468</v>
       </c>
       <c r="J9" t="n">
-        <v>12055</v>
+        <v>11864</v>
       </c>
       <c r="K9" t="n">
-        <v>26167</v>
+        <v>61604</v>
       </c>
       <c r="L9" t="n">
-        <v>1.61</v>
+        <v>4.23</v>
       </c>
       <c r="M9" t="n">
-        <v>1.19</v>
+        <v>0.88</v>
       </c>
       <c r="N9" t="n">
-        <v>24.38</v>
+        <v>43.61</v>
       </c>
       <c r="O9" t="n">
-        <v>61.4</v>
+        <v>16.91</v>
       </c>
       <c r="P9" t="n">
-        <v>24.66</v>
+        <v>9.33</v>
       </c>
       <c r="Q9" t="n">
-        <v>4719</v>
+        <v>4815</v>
       </c>
       <c r="R9" t="n">
-        <v>-144</v>
+        <v>-25477</v>
       </c>
       <c r="S9" t="n">
-        <v>-4073</v>
+        <v>18337</v>
       </c>
       <c r="T9" t="n">
-        <v>4597</v>
+        <v>4693</v>
       </c>
       <c r="U9" t="n">
         <v>122</v>
       </c>
       <c r="V9" t="n">
-        <v>-44</v>
+        <v>-48</v>
       </c>
       <c r="W9" t="n">
-        <v>1358</v>
+        <v>2308</v>
       </c>
       <c r="X9" t="n">
-        <v>5076</v>
+        <v>6125</v>
       </c>
       <c r="Y9" t="n">
-        <v>10988</v>
+        <v>6823</v>
       </c>
       <c r="Z9" t="n">
-        <v>35.34</v>
+        <v>49.98</v>
       </c>
       <c r="AA9" t="n">
-        <v>13163</v>
+        <v>40170</v>
       </c>
       <c r="AB9" t="n">
-        <v>14379</v>
+        <v>12809</v>
       </c>
       <c r="AC9" t="n">
-        <v>4.6</v>
+        <v>5.39</v>
       </c>
       <c r="AD9" t="n">
-        <v>57.55</v>
+        <v>183.77</v>
       </c>
       <c r="AE9" t="n">
-        <v>1707</v>
+        <v>7176</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>45047</v>
+      <c r="A10" s="2" t="n">
+        <v>45139</v>
       </c>
       <c r="B10" t="n">
-        <v>92.76000000000001</v>
+        <v>111.48</v>
       </c>
       <c r="C10" t="n">
-        <v>25.12</v>
+        <v>27.17</v>
       </c>
       <c r="D10" t="n">
-        <v>3.98</v>
+        <v>3.68</v>
       </c>
       <c r="E10" t="n">
-        <v>4137</v>
+        <v>3978</v>
       </c>
       <c r="F10" t="n">
-        <v>39.86</v>
+        <v>37.21</v>
       </c>
       <c r="G10" t="n">
-        <v>14.67</v>
+        <v>16.68</v>
       </c>
       <c r="H10" t="n">
-        <v>322911500</v>
+        <v>368230800</v>
       </c>
       <c r="I10" t="n">
-        <v>38194</v>
+        <v>38222</v>
       </c>
       <c r="J10" t="n">
-        <v>11553</v>
+        <v>12055</v>
       </c>
       <c r="K10" t="n">
-        <v>26641</v>
+        <v>26167</v>
       </c>
       <c r="L10" t="n">
-        <v>1.69</v>
+        <v>1.61</v>
       </c>
       <c r="M10" t="n">
-        <v>1.21</v>
+        <v>1.19</v>
       </c>
       <c r="N10" t="n">
-        <v>22.18</v>
+        <v>24.33</v>
       </c>
       <c r="O10" t="n">
-        <v>58.02</v>
+        <v>61.4</v>
       </c>
       <c r="P10" t="n">
-        <v>24.05</v>
+        <v>24.66</v>
       </c>
       <c r="Q10" t="n">
-        <v>4502</v>
+        <v>4719</v>
       </c>
       <c r="R10" t="n">
-        <v>-318</v>
+        <v>-144</v>
       </c>
       <c r="S10" t="n">
-        <v>-5278</v>
+        <v>-4073</v>
       </c>
       <c r="T10" t="n">
-        <v>4380</v>
+        <v>4597</v>
       </c>
       <c r="U10" t="n">
         <v>122</v>
       </c>
       <c r="V10" t="n">
-        <v>-94</v>
+        <v>-44</v>
       </c>
       <c r="W10" t="n">
-        <v>1312</v>
+        <v>1358</v>
       </c>
       <c r="X10" t="n">
-        <v>4929</v>
+        <v>5076</v>
       </c>
       <c r="Y10" t="n">
-        <v>10360</v>
+        <v>10988</v>
       </c>
       <c r="Z10" t="n">
-        <v>37.39</v>
+        <v>35.34</v>
       </c>
       <c r="AA10" t="n">
-        <v>11956</v>
+        <v>13163</v>
       </c>
       <c r="AB10" t="n">
-        <v>13887</v>
+        <v>14379</v>
       </c>
       <c r="AC10" t="n">
-        <v>4.61</v>
+        <v>4.6</v>
       </c>
       <c r="AD10" t="n">
-        <v>54.98</v>
+        <v>57.55</v>
       </c>
       <c r="AE10" t="n">
-        <v>2806</v>
+        <v>1707</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>44958</v>
+      <c r="A11" s="2" t="n">
+        <v>45047</v>
       </c>
       <c r="B11" t="n">
-        <v>62.93</v>
+        <v>92.56</v>
       </c>
       <c r="C11" t="n">
-        <v>20</v>
+        <v>25.06</v>
       </c>
       <c r="D11" t="n">
-        <v>5</v>
+        <v>3.99</v>
       </c>
       <c r="E11" t="n">
-        <v>4230</v>
+        <v>4137</v>
       </c>
       <c r="F11" t="n">
-        <v>42.33</v>
+        <v>39.86</v>
       </c>
       <c r="G11" t="n">
-        <v>10.19</v>
+        <v>14.64</v>
       </c>
       <c r="H11" t="n">
-        <v>237507600</v>
+        <v>322206000</v>
       </c>
       <c r="I11" t="n">
-        <v>38167</v>
+        <v>38194</v>
       </c>
       <c r="J11" t="n">
-        <v>12647</v>
+        <v>11553</v>
       </c>
       <c r="K11" t="n">
-        <v>25520</v>
+        <v>26641</v>
       </c>
       <c r="L11" t="n">
-        <v>1.72</v>
+        <v>1.69</v>
       </c>
       <c r="M11" t="n">
-        <v>1.09</v>
+        <v>1.21</v>
       </c>
       <c r="N11" t="n">
-        <v>17.69</v>
+        <v>22.13</v>
       </c>
       <c r="O11" t="n">
-        <v>50.13</v>
+        <v>58.02</v>
       </c>
       <c r="P11" t="n">
-        <v>22.12</v>
+        <v>24.05</v>
       </c>
       <c r="Q11" t="n">
-        <v>4036</v>
+        <v>4502</v>
       </c>
       <c r="R11" t="n">
-        <v>-103</v>
+        <v>-318</v>
       </c>
       <c r="S11" t="n">
-        <v>-3702</v>
+        <v>-5278</v>
       </c>
       <c r="T11" t="n">
-        <v>3933</v>
+        <v>4380</v>
       </c>
       <c r="U11" t="n">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="V11" t="n">
-        <v>-122</v>
+        <v>-94</v>
       </c>
       <c r="W11" t="n">
-        <v>1195</v>
+        <v>1312</v>
       </c>
       <c r="X11" t="n">
-        <v>4795</v>
+        <v>4929</v>
       </c>
       <c r="Y11" t="n">
-        <v>11353</v>
+        <v>10360</v>
       </c>
       <c r="Z11" t="n">
-        <v>43.75</v>
+        <v>37.39</v>
       </c>
       <c r="AA11" t="n">
-        <v>9977</v>
+        <v>11956</v>
       </c>
       <c r="AB11" t="n">
-        <v>13063</v>
+        <v>13887</v>
       </c>
       <c r="AC11" t="n">
         <v>4.61</v>
       </c>
       <c r="AD11" t="n">
-        <v>51.03</v>
+        <v>54.98</v>
       </c>
       <c r="AE11" t="n">
-        <v>1188</v>
+        <v>2806</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>44774</v>
+      <c r="A12" s="2" t="n">
+        <v>44958</v>
       </c>
       <c r="B12" t="n">
-        <v>63.38</v>
+        <v>62.8</v>
       </c>
       <c r="C12" t="n">
-        <v>19.75</v>
+        <v>19.96</v>
       </c>
       <c r="D12" t="n">
-        <v>5.06</v>
+        <v>5.01</v>
       </c>
       <c r="E12" t="n">
-        <v>3866</v>
+        <v>4230</v>
       </c>
       <c r="F12" t="n">
-        <v>35.43</v>
+        <v>42.33</v>
       </c>
       <c r="G12" t="n">
-        <v>9.1</v>
+        <v>10.17</v>
       </c>
       <c r="H12" t="n">
-        <v>190066500</v>
+        <v>237006000</v>
       </c>
       <c r="I12" t="n">
-        <v>39191</v>
+        <v>38167</v>
       </c>
       <c r="J12" t="n">
+        <v>12647</v>
+      </c>
+      <c r="K12" t="n">
+        <v>25520</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="N12" t="n">
+        <v>17.66</v>
+      </c>
+      <c r="O12" t="n">
+        <v>50.13</v>
+      </c>
+      <c r="P12" t="n">
+        <v>22.12</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>4036</v>
+      </c>
+      <c r="R12" t="n">
+        <v>-103</v>
+      </c>
+      <c r="S12" t="n">
+        <v>-3702</v>
+      </c>
+      <c r="T12" t="n">
+        <v>3933</v>
+      </c>
+      <c r="U12" t="n">
+        <v>103</v>
+      </c>
+      <c r="V12" t="n">
+        <v>-122</v>
+      </c>
+      <c r="W12" t="n">
+        <v>1195</v>
+      </c>
+      <c r="X12" t="n">
+        <v>4795</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>11353</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>43.75</v>
+      </c>
+      <c r="AA12" t="n">
         <v>9977</v>
       </c>
-      <c r="K12" t="n">
-        <v>29214</v>
-      </c>
-      <c r="L12" t="n">
-        <v>2.26</v>
-      </c>
-      <c r="M12" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="N12" t="n">
-        <v>17</v>
-      </c>
-      <c r="O12" t="n">
-        <v>46.53</v>
-      </c>
-      <c r="P12" t="n">
-        <v>19.71</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>4424</v>
-      </c>
-      <c r="R12" t="n">
-        <v>80</v>
-      </c>
-      <c r="S12" t="n">
-        <v>-3532</v>
-      </c>
-      <c r="T12" t="n">
-        <v>4308</v>
-      </c>
-      <c r="U12" t="n">
-        <v>116</v>
-      </c>
-      <c r="V12" t="n">
-        <v>-117</v>
-      </c>
-      <c r="W12" t="n">
-        <v>1255</v>
-      </c>
-      <c r="X12" t="n">
-        <v>4810</v>
-      </c>
-      <c r="Y12" t="n">
-        <v>8859</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>43.16</v>
-      </c>
-      <c r="AA12" t="n">
-        <v>9115</v>
-      </c>
       <c r="AB12" t="n">
-        <v>11208</v>
+        <v>13063</v>
       </c>
       <c r="AC12" t="n">
-        <v>4.29</v>
+        <v>4.61</v>
       </c>
       <c r="AD12" t="n">
-        <v>57.89</v>
+        <v>51.03</v>
       </c>
       <c r="AE12" t="n">
-        <v>1500</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>44682</v>
+      <c r="A13" s="2" t="n">
+        <v>44774</v>
       </c>
       <c r="B13" t="n">
-        <v>87.76000000000001</v>
+        <v>63.24</v>
       </c>
       <c r="C13" t="n">
-        <v>27.3</v>
+        <v>19.71</v>
       </c>
       <c r="D13" t="n">
-        <v>3.66</v>
+        <v>5.07</v>
       </c>
       <c r="E13" t="n">
-        <v>3529</v>
+        <v>3866</v>
       </c>
       <c r="F13" t="n">
-        <v>31.04</v>
+        <v>35.43</v>
       </c>
       <c r="G13" t="n">
-        <v>10.53</v>
+        <v>9.08</v>
       </c>
       <c r="H13" t="n">
-        <v>220728000</v>
+        <v>189661500</v>
       </c>
       <c r="I13" t="n">
-        <v>39164</v>
+        <v>39191</v>
       </c>
       <c r="J13" t="n">
-        <v>9005</v>
+        <v>9977</v>
       </c>
       <c r="K13" t="n">
-        <v>30159</v>
+        <v>29214</v>
       </c>
       <c r="L13" t="n">
-        <v>2.71</v>
+        <v>2.26</v>
       </c>
       <c r="M13" t="n">
-        <v>1.44</v>
+        <v>1.4</v>
       </c>
       <c r="N13" t="n">
-        <v>22.52</v>
+        <v>16.97</v>
       </c>
       <c r="O13" t="n">
-        <v>38.79</v>
+        <v>46.53</v>
       </c>
       <c r="P13" t="n">
-        <v>17.21</v>
+        <v>19.71</v>
       </c>
       <c r="Q13" t="n">
-        <v>4243</v>
+        <v>4424</v>
       </c>
       <c r="R13" t="n">
-        <v>-310</v>
+        <v>80</v>
       </c>
       <c r="S13" t="n">
-        <v>-5147</v>
+        <v>-3532</v>
       </c>
       <c r="T13" t="n">
-        <v>4158</v>
+        <v>4308</v>
       </c>
       <c r="U13" t="n">
-        <v>85</v>
+        <v>116</v>
       </c>
       <c r="V13" t="n">
-        <v>-111</v>
+        <v>-117</v>
       </c>
       <c r="W13" t="n">
-        <v>1261</v>
+        <v>1255</v>
       </c>
       <c r="X13" t="n">
-        <v>4799</v>
+        <v>4810</v>
       </c>
       <c r="Y13" t="n">
-        <v>7900</v>
+        <v>8859</v>
       </c>
       <c r="Z13" t="n">
-        <v>48.71</v>
+        <v>43.16</v>
       </c>
       <c r="AA13" t="n">
-        <v>6053</v>
+        <v>9115</v>
       </c>
       <c r="AB13" t="n">
-        <v>9714</v>
+        <v>11208</v>
       </c>
       <c r="AC13" t="n">
         <v>4.29</v>
       </c>
       <c r="AD13" t="n">
-        <v>69.58</v>
+        <v>57.89</v>
       </c>
       <c r="AE13" t="n">
-        <v>2776</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>44593</v>
+      <c r="A14" s="2" t="n">
+        <v>44682</v>
       </c>
       <c r="B14" t="n">
-        <v>93.5</v>
+        <v>87.59</v>
       </c>
       <c r="C14" t="n">
-        <v>32.28</v>
+        <v>27.24</v>
       </c>
       <c r="D14" t="n">
-        <v>3.1</v>
+        <v>3.67</v>
       </c>
       <c r="E14" t="n">
-        <v>3244</v>
+        <v>3529</v>
       </c>
       <c r="F14" t="n">
-        <v>31.12</v>
+        <v>31.04</v>
       </c>
       <c r="G14" t="n">
-        <v>9.76</v>
+        <v>10.51</v>
       </c>
       <c r="H14" t="n">
-        <v>224210400</v>
+        <v>220279200</v>
       </c>
       <c r="I14" t="n">
-        <v>39205</v>
+        <v>39164</v>
       </c>
       <c r="J14" t="n">
-        <v>10219</v>
+        <v>9005</v>
       </c>
       <c r="K14" t="n">
-        <v>28986</v>
+        <v>30159</v>
       </c>
       <c r="L14" t="n">
-        <v>3.02</v>
+        <v>2.71</v>
       </c>
       <c r="M14" t="n">
-        <v>1.26</v>
+        <v>1.44</v>
       </c>
       <c r="N14" t="n">
-        <v>26.41</v>
+        <v>22.48</v>
       </c>
       <c r="O14" t="n">
-        <v>30.13</v>
+        <v>38.79</v>
       </c>
       <c r="P14" t="n">
-        <v>14.45</v>
+        <v>17.21</v>
       </c>
       <c r="Q14" t="n">
-        <v>3486</v>
+        <v>4243</v>
       </c>
       <c r="R14" t="n">
-        <v>-309</v>
+        <v>-310</v>
       </c>
       <c r="S14" t="n">
-        <v>-5121</v>
+        <v>-5147</v>
       </c>
       <c r="T14" t="n">
-        <v>3385</v>
+        <v>4158</v>
       </c>
       <c r="U14" t="n">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="V14" t="n">
-        <v>-85</v>
+        <v>-111</v>
       </c>
       <c r="W14" t="n">
-        <v>1206</v>
+        <v>1261</v>
       </c>
       <c r="X14" t="n">
-        <v>4775</v>
+        <v>4799</v>
       </c>
       <c r="Y14" t="n">
-        <v>9054</v>
+        <v>7900</v>
       </c>
       <c r="Z14" t="n">
-        <v>61.02999999999999</v>
+        <v>48.71</v>
       </c>
       <c r="AA14" t="n">
-        <v>5215</v>
+        <v>6053</v>
       </c>
       <c r="AB14" t="n">
-        <v>7700</v>
+        <v>9714</v>
       </c>
       <c r="AC14" t="n">
-        <v>4.28</v>
+        <v>4.29</v>
       </c>
       <c r="AD14" t="n">
-        <v>73.56</v>
+        <v>69.58</v>
       </c>
       <c r="AE14" t="n">
-        <v>2724</v>
+        <v>2776</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>44409</v>
+      <c r="A15" s="2" t="n">
+        <v>44593</v>
       </c>
       <c r="B15" t="n">
-        <v>103.62</v>
+        <v>93.29000000000001</v>
       </c>
       <c r="C15" t="n">
-        <v>36.17</v>
+        <v>32.21</v>
       </c>
       <c r="D15" t="n">
-        <v>2.76</v>
+        <v>3.1</v>
       </c>
       <c r="E15" t="n">
-        <v>2260</v>
+        <v>3244</v>
       </c>
       <c r="F15" t="n">
-        <v>26.59</v>
+        <v>31.12</v>
       </c>
       <c r="G15" t="n">
-        <v>7.67</v>
+        <v>9.74</v>
       </c>
       <c r="H15" t="n">
-        <v>186717300</v>
+        <v>223716000</v>
       </c>
       <c r="I15" t="n">
-        <v>40178</v>
+        <v>39205</v>
       </c>
       <c r="J15" t="n">
-        <v>11105</v>
+        <v>10219</v>
       </c>
       <c r="K15" t="n">
-        <v>29073</v>
+        <v>28986</v>
       </c>
       <c r="L15" t="n">
-        <v>3.88</v>
+        <v>3.02</v>
       </c>
       <c r="M15" t="n">
-        <v>1.19</v>
+        <v>1.26</v>
       </c>
       <c r="N15" t="n">
-        <v>28.81</v>
+        <v>26.36</v>
       </c>
       <c r="O15" t="n">
-        <v>21.11</v>
+        <v>30.13</v>
       </c>
       <c r="P15" t="n">
-        <v>11.15</v>
+        <v>14.45</v>
       </c>
       <c r="Q15" t="n">
-        <v>3541</v>
+        <v>3486</v>
       </c>
       <c r="R15" t="n">
-        <v>-47</v>
+        <v>-309</v>
       </c>
       <c r="S15" t="n">
-        <v>-1907</v>
+        <v>-5121</v>
       </c>
       <c r="T15" t="n">
-        <v>3426</v>
+        <v>3385</v>
       </c>
       <c r="U15" t="n">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="V15" t="n">
-        <v>-83</v>
+        <v>-85</v>
       </c>
       <c r="W15" t="n">
-        <v>1205</v>
+        <v>1206</v>
       </c>
       <c r="X15" t="n">
-        <v>4799</v>
+        <v>4775</v>
       </c>
       <c r="Y15" t="n">
-        <v>9135</v>
+        <v>9054</v>
       </c>
       <c r="Z15" t="n">
-        <v>70.82000000000001</v>
+        <v>61.02999999999999</v>
       </c>
       <c r="AA15" t="n">
-        <v>5224</v>
+        <v>5215</v>
       </c>
       <c r="AB15" t="n">
-        <v>6734</v>
+        <v>7700</v>
       </c>
       <c r="AC15" t="n">
-        <v>3.79</v>
+        <v>4.28</v>
       </c>
       <c r="AD15" t="n">
-        <v>86.34999999999999</v>
+        <v>73.56</v>
       </c>
       <c r="AE15" t="n">
-        <v>0</v>
+        <v>2724</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>44317</v>
+      <c r="A16" s="2" t="n">
+        <v>44409</v>
       </c>
       <c r="B16" t="n">
-        <v>123.59</v>
+        <v>103.41</v>
       </c>
       <c r="C16" t="n">
-        <v>45.55</v>
+        <v>36.1</v>
       </c>
       <c r="D16" t="n">
-        <v>2.2</v>
+        <v>2.77</v>
       </c>
       <c r="E16" t="n">
-        <v>2108</v>
+        <v>2260</v>
       </c>
       <c r="F16" t="n">
-        <v>21.44</v>
+        <v>26.59</v>
       </c>
       <c r="G16" t="n">
-        <v>7.32</v>
+        <v>7.66</v>
       </c>
       <c r="H16" t="n">
-        <v>175133800</v>
+        <v>186347400</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>40178</v>
       </c>
       <c r="J16" t="n">
-        <v>9518</v>
+        <v>11105</v>
       </c>
       <c r="K16" t="n">
-        <v>-9518</v>
+        <v>29073</v>
       </c>
       <c r="L16" t="n">
-        <v>-1.55</v>
+        <v>3.88</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.4</v>
+        <v>1.19</v>
       </c>
       <c r="N16" t="n">
-        <v>30.06</v>
+        <v>28.76</v>
       </c>
       <c r="O16" t="n">
-        <v>15.97</v>
+        <v>21.11</v>
       </c>
       <c r="P16" t="n">
-        <v>24.4</v>
+        <v>11.15</v>
       </c>
       <c r="Q16" t="n">
-        <v>3569</v>
+        <v>3541</v>
       </c>
       <c r="R16" t="n">
-        <v>-126</v>
+        <v>-47</v>
       </c>
       <c r="S16" t="n">
-        <v>-3477</v>
+        <v>-1907</v>
       </c>
       <c r="T16" t="n">
-        <v>3443</v>
+        <v>3426</v>
       </c>
       <c r="U16" t="n">
-        <v>126</v>
+        <v>115</v>
       </c>
       <c r="V16" t="n">
-        <v>-63</v>
+        <v>-83</v>
       </c>
       <c r="W16" t="n">
-        <v>1238</v>
+        <v>1205</v>
       </c>
       <c r="X16" t="n">
-        <v>4883</v>
+        <v>4799</v>
       </c>
       <c r="Y16" t="n">
-        <v>7809</v>
+        <v>9135</v>
       </c>
       <c r="Z16" t="n">
-        <v>82.45</v>
+        <v>70.82000000000001</v>
       </c>
       <c r="AA16" t="n">
-        <v>4267</v>
+        <v>5224</v>
       </c>
       <c r="AB16" t="n">
-        <v>5715</v>
+        <v>6734</v>
       </c>
       <c r="AC16" t="n">
         <v>3.79</v>
       </c>
       <c r="AD16" t="n">
-        <v>109.53</v>
+        <v>86.34999999999999</v>
       </c>
       <c r="AE16" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>44228</v>
+      <c r="A17" s="2" t="n">
+        <v>44317</v>
       </c>
       <c r="B17" t="n">
-        <v>131.93</v>
+        <v>123.34</v>
       </c>
       <c r="C17" t="n">
-        <v>62.9</v>
+        <v>45.46</v>
       </c>
       <c r="D17" t="n">
-        <v>1.59</v>
+        <v>2.2</v>
       </c>
       <c r="E17" t="n">
-        <v>1975</v>
+        <v>2108</v>
       </c>
       <c r="F17" t="n">
-        <v>19.59</v>
+        <v>21.44</v>
       </c>
       <c r="G17" t="n">
-        <v>7.18</v>
+        <v>7.3</v>
       </c>
       <c r="H17" t="n">
-        <v>172038900</v>
+        <v>174765700</v>
       </c>
       <c r="I17" t="n">
-        <v>41068</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>9552</v>
+        <v>9518</v>
       </c>
       <c r="K17" t="n">
-        <v>31516</v>
+        <v>-9518</v>
       </c>
       <c r="L17" t="n">
-        <v>6.44</v>
+        <v>-1.55</v>
       </c>
       <c r="M17" t="n">
-        <v>1.31</v>
+        <v>-0.4</v>
       </c>
       <c r="N17" t="n">
-        <v>41.59</v>
+        <v>30</v>
       </c>
       <c r="O17" t="n">
-        <v>11.33</v>
+        <v>15.97</v>
       </c>
       <c r="P17" t="n">
-        <v>7.15</v>
+        <v>24.4</v>
       </c>
       <c r="Q17" t="n">
-        <v>3113</v>
+        <v>3569</v>
       </c>
       <c r="R17" t="n">
-        <v>-122</v>
+        <v>-126</v>
       </c>
       <c r="S17" t="n">
-        <v>-1057</v>
+        <v>-3477</v>
       </c>
       <c r="T17" t="n">
-        <v>2999</v>
+        <v>3443</v>
       </c>
       <c r="U17" t="n">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="V17" t="n">
-        <v>-94</v>
+        <v>-63</v>
       </c>
       <c r="W17" t="n">
-        <v>1211</v>
+        <v>1238</v>
       </c>
       <c r="X17" t="n">
-        <v>4903</v>
+        <v>4883</v>
       </c>
       <c r="Y17" t="n">
-        <v>7606</v>
+        <v>7809</v>
       </c>
       <c r="Z17" t="n">
-        <v>112.47</v>
+        <v>82.45</v>
       </c>
       <c r="AA17" t="n">
-        <v>15176</v>
+        <v>4267</v>
       </c>
       <c r="AB17" t="n">
-        <v>4073</v>
+        <v>5715</v>
       </c>
       <c r="AC17" t="n">
         <v>3.79</v>
       </c>
       <c r="AD17" t="n">
+        <v>109.53</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>44228</v>
+      </c>
+      <c r="B18" t="n">
+        <v>131.65</v>
+      </c>
+      <c r="C18" t="n">
+        <v>62.77</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1975</v>
+      </c>
+      <c r="F18" t="n">
+        <v>19.59</v>
+      </c>
+      <c r="G18" t="n">
+        <v>7.16</v>
+      </c>
+      <c r="H18" t="n">
+        <v>171672600</v>
+      </c>
+      <c r="I18" t="n">
+        <v>41068</v>
+      </c>
+      <c r="J18" t="n">
+        <v>9552</v>
+      </c>
+      <c r="K18" t="n">
+        <v>31516</v>
+      </c>
+      <c r="L18" t="n">
+        <v>6.44</v>
+      </c>
+      <c r="M18" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="N18" t="n">
+        <v>41.52</v>
+      </c>
+      <c r="O18" t="n">
+        <v>11.33</v>
+      </c>
+      <c r="P18" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>3113</v>
+      </c>
+      <c r="R18" t="n">
+        <v>-122</v>
+      </c>
+      <c r="S18" t="n">
+        <v>-1057</v>
+      </c>
+      <c r="T18" t="n">
+        <v>2999</v>
+      </c>
+      <c r="U18" t="n">
+        <v>114</v>
+      </c>
+      <c r="V18" t="n">
+        <v>-94</v>
+      </c>
+      <c r="W18" t="n">
+        <v>1211</v>
+      </c>
+      <c r="X18" t="n">
+        <v>4903</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>7606</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>112.47</v>
+      </c>
+      <c r="AA18" t="n">
+        <v>15176</v>
+      </c>
+      <c r="AB18" t="n">
+        <v>4073</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="AD18" t="n">
         <v>118.33</v>
       </c>
-      <c r="AE17" t="n">
+      <c r="AE18" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>